<commit_message>
docs: verify future-work tracker against code — 6 done, 10 partial, 35 open
Audited all 51 items against code/edge-fns/migrations/git. Corrected Hub drift:
6 items already DONE (voice route-move, native CPL prod, payments build,
subscription field fix, workspace mis-route guard, native toolbar on prod);
10 PARTIAL with named remainder; 35 genuinely open. Status + evidence per row.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-2026-07-05.xlsx
+++ b/docs/CrewLogic-Future-Work-2026-07-05.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +39,19 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <color rgb="009C3A3A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E7A34"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -59,7 +70,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -106,14 +132,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -496,7 +531,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic - Identified Future Work (from .HUB/Hub.md) - 2026-07-05</t>
+          <t>CrewLogic - Future Work (from .HUB/Hub.md) - verified against code 2026-07-05  |  6 Done, 10 Partial, 35 Not started</t>
         </is>
       </c>
     </row>
@@ -567,36 +602,52 @@
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Receiver deployed; live path unexercised — prod Linxup franchise 209f31ef cameras offline (hardware-blocked).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Telematics / Trucks</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Linxup job-level arrive/leave matching</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Phase-1 covers fence-name alerts only, not job-level arrive/leave.</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Needs Linxup geofence-create; explicit follow-on.</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>crewlogic-geofence-create hard-rejects non-Motive (index.ts:130); Linxup geofence-create not built.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -623,36 +674,52 @@
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Owner action — per-franchise Vault token doesn't carry dev-&gt;prod; re-enter #90 Motive token in prod Settings.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Telematics / Trucks</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Refine dashcam/fault-code event labels</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Geofence alerts auto-capture dashcam-disconnect and fault-code events generically.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Refine the labels when each type is first seen live.</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>crewlogic-motive-webhook stores fault/dashcam events generically (index.ts:116); refine labels when first seen.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -679,36 +746,52 @@
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>No on-site-count code exists (grep clean); deferred.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Telematics / Trucks</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Telematics partnership / referral links</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Explore a Motive/Linxup referral deal since CrewLogic funnels GPS signups.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Hook in place (plain vendor links); swap for referral URLs when they exist.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Links still plain gomotive.com/linxup.com (index.html:7854-55,11271-72); owner business action.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -735,36 +818,52 @@
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Estimates Desk shipped w/o iCal; no .ics/VEVENT code anywhere.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Maps / Dispatch / Routing</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Per-appointment Vonigo cancel</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Cancelling one appointment on a multi-appointment Vonigo job currently just blocks, since per-appointment WO-cancel isn't achievable by API probing.</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Parked pending a Vonigo support ticket; wire the correct cancel-by-woID call when they return it.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Multi-appt cancel still blocks + routes to Vonigo grid; cancel-by-woID not wired (Vonigo ticket pending).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -791,36 +890,52 @@
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Geocoded server tools EXIST (crewlogic-dispatch geocode/listRouteJobs/suggestSlots/moveJob); cross-route recombine engine not built.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Maps / Dispatch / Routing</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>In-app reschedule ('pull it forward')</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Move a job's appointment from inside CrewLogic when a truck is near a job scheduled days out.</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Not started; needs open-slot visibility, a date/time picker on the job popup, and a Vonigo WorkOrder write.</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Desktop drag-to-move across days + voice move work; no date/time reschedule picker on the job popup.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -847,36 +962,52 @@
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>None shipped: disposalWait still static global; no sheet import; no AI cost-vs-time rec; recycling/donation hours not mirrored.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Maps / Dispatch / Routing</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Route Optimizer multi-tenant re-architecture</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>The #90 route engine still runs on n8n + the owner's personal Google Sheet and is hard-gated to franchise 90.</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Move to edge functions + Supabase tables before any other franchisee (blocks it as a paid Enterprise feature).</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>optimizeRoute() still calls n8n /crewlogic-route (index.html:11598); not migrated to edge fns/tables.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -903,36 +1034,52 @@
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Single global disposalWait; facilities table (0023) has no wait column; no per-site input.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Maps / Dispatch / Routing</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Weather alerts: narrow scope + trucks screen</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>NWS weather alerts are state-level and shown only on the dashboard + Job Plan.</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Narrow to the office point; surface on the trucks screen.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>crewlogic-weather is state-level; dashboard + Job Plan only; not narrowed to office point, not on trucks screen.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -959,36 +1106,52 @@
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE — voice move-with-route shipped (crewlogic-dispatch -&gt; Vonigo method16; dispatch/index.ts:453,522).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Maps / Dispatch / Routing</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Voice Dispatcher: prod write + voice-bar popup</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>The Voice AI Dispatcher is live, but the move/cancel/duration WRITE path is only read-verified.</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Owner runs a real command; also mirror the unified conversation popup on the Manage Jobs voice bar.</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Write path fully wired (execute-&gt;method16 move/cancel/duration) but NOT prod-write-verified (dev VONIGO_READONLY); unified popup not mirrored on Manage Jobs voice bar.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1015,36 +1178,52 @@
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>townFromAddress returns raw UPPERCASE Vonigo segment (job-geofence-sync:123); title-case tweak.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Pricing / CRM / Vonigo</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Vonigo date-range CRM pipeline</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Pull leads, estimates, cancellations, cases, and UCBs from Vonigo by date range into a CRM-style pipeline so nothing slips.</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Not started; open questions: define 'UCB,' endpoint mapping per category, pull cadence.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>No date-range CRM pipeline; only crewlogic-todays-workorders (today-only). Bigger project.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1071,36 +1250,52 @@
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Vonigo write path proven, but simplify-prompt + nightly cron not built; no NA/summary cron.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Pricing / CRM / Vonigo</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Vonigo submit server-side null-price guard</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>v5.49.1 added the frontend guard that auto-heals/aborts on charges missing a priceItemID.</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Optional server-side guard in crewlogic-estimate deferred.</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="7" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Frontend guard live (v5.49.1); handleSubmitQuote has NO server-side null-priceItemID rejection — server guard deferred.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1127,36 +1322,52 @@
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE — CPL fix on main (v5.50.0, f0c32f7) + prod crewlogic-pricing returns blockType (downloaded+checked). Hub 'pending' was stale.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Pricing / CRM / Vonigo</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Shed/building estimator undercounts volume</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>The shed/building volume estimator computes ~half the actual volume.</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Not started; add floor-joist depth, roof-joist depth, and shingle-layer inputs, verified against a known shed.</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>calcShed still uses ~half-volume formula w/ no joist/shingle inputs (index.html ~23508).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1183,36 +1394,52 @@
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Four buttons still hardcode 16 cy (index.html 3457,3466,3607,3616). Cosmetic.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Native mode / Onboarding</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Onboarding: serviceStates + estimator default state</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Capture the franchise's serviceStates and a per-estimator default state at signup/provisioning, owner-editable in Settings.</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Not started; feeds Town Price Lookup.</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>serviceStates captured/editable + feeds Town Price Lookup; per-estimator default state parked + signup-time capture not started.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1239,36 +1466,52 @@
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>No first-run empty-state prompt (add ZIPs/import customers) exists.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Native mode / Onboarding</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Native price-book onboarding finishers</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>The 'set up your price book' prompt is partly done.</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>Pending: the orange home Price Lookup tile for price-book-less native owners (needs a hasPriceBook signal) + the empty-default-list UX.</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="7" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Friendly 'no price book' notice DONE; orange home Price Lookup tile NOT built (no hasPriceBook signal).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1295,36 +1538,52 @@
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Two-URL split done/live; Phase 2 onboarding wizard has no code.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Settings / UX</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Streamline the Settings environment</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>Owner: 'the whole settings environment is a mess, need to streamline it... later.'</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>A bigger UX/reorg pass; not started.</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr"/>
-      <c r="G30" s="7" t="inlineStr"/>
-      <c r="H30" s="7" t="inlineStr"/>
+      <c r="F30" s="8" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>No Settings reorg done; owner backlog 'the whole settings environment is a mess... later.'</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1351,36 +1610,52 @@
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Reorder IS live (SortableJS, 0021); HIDE logic does not exist.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Settings / UX</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>index.html size / architecture review</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>The single ~22k-line index.html keeps growing.</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
         <is>
           <t>Deliberate keep-single-file vs light-split/build decision; queued for strategy mode; any split must preserve the no-build Cloudflare Pages deploy.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr"/>
-      <c r="G32" s="7" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Decision not made; file ~22k lines; keep-single-file vs split undecided.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1407,36 +1682,52 @@
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE (build) — billing built + shipped DORMANT: crewlogic-billing (Stripe checkout/portal/webhook), paywall tier picker, migrations 0025/0026. Hub 'build not started' was WRONG. Activation = item #39.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Payments / Billing</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Billing activation</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>Round-1 billing shipped to prod dormant (BILLING_ENABLED off).</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>Apply migration 0025 to prod + set up LIVE-mode Stripe before flipping BILLING_ENABLED (then ENFORCE_TRIAL).</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr"/>
-      <c r="G34" s="7" t="inlineStr"/>
-      <c r="H34" s="7" t="inlineStr"/>
+      <c r="F34" s="8" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Dormant by design — BILLING_ENABLED=IS_DEV_ENV (prod OFF); flip + LIVE Stripe + apply 0025 to prod remain.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1463,36 +1754,52 @@
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE (superseded) — gate logic now never lets 'free' tier override an access-granting tenant (index.html:5316, oauth-callback:490); provisionNative writes null intentionally. 'Write free' ask moot.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n">
+      <c r="A36" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Payments / Billing</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Trial-expiry UX questions</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t>Parked: what happens at 14-day trial end, messaging, lockout, re-enable without losing settings.</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>Code read suggests ENFORCE_TRIAL is currently false and settings persist; verify before answering definitively.</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr"/>
-      <c r="G36" s="7" t="inlineStr"/>
-      <c r="H36" s="7" t="inlineStr"/>
+      <c r="F36" s="8" t="inlineStr"/>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Countdown banner + trialState shipped (non-blocking copy); ENFORCE_TRIAL=false — end-of-trial lockout/re-enable UX decisions remain.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -1519,36 +1826,52 @@
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>One silent refresh then clean re-auth redirect; no soft 'Reconnecting...' banner / one-tap re-auth.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
+      <c r="A38" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>Auth / Session</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Harden crewlogic-trucks caller verification</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
         <is>
           <t>Per-request caller verification is deferred because Google-OAuth owners have no Supabase JWT.</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Folded into future unified-auth work; residual risk low.</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr"/>
-      <c r="G38" s="7" t="inlineStr"/>
-      <c r="H38" s="7" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>crewlogic-trucks uses service-role RPC, CORS '*', no per-request caller/JWT/ownership check.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -1575,36 +1898,52 @@
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE — showNameWorkspaceScreen only on no-profile+no-invite; buildSessionFromSupabaseAuth retries once on incomplete profile.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n">
+      <c r="A40" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>Auth / Session</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Native toolbar-fix prod promote</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
         <is>
           <t>The native-estimate reopen toolbar bug is fixed and owner-verified on dev.</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>Pending prod promote.</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr"/>
-      <c r="G40" s="7" t="inlineStr"/>
-      <c r="H40" s="7" t="inlineStr"/>
+      <c r="F40" s="8" t="inlineStr"/>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED DONE — renderChargeRows-&gt;renderCharges fix on MAIN at v5.50.0 (836f993). Hub 'pending prod promote' was stale.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -1631,36 +1970,52 @@
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Both still Eastern-hardcoded: todays-workorders getEasternMidnightEpoch + job-plan nowET; no resolveTimezone/STATE_TZ.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>Multi-tenant / Time zones</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>Onboarding: capture location + confirm timezone</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>Have the franchisee enter full office location and confirm their IANA timezone at onboarding (cost_settings.officeTimezone).</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>Not started; until then each non-ET franchise needs a manual officeTimezone backfill.</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr"/>
-      <c r="G42" s="7" t="inlineStr"/>
-      <c r="H42" s="7" t="inlineStr"/>
+      <c r="F42" s="8" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>officeTimezone only READ, never written; onboarding/settings capture officeState only.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -1687,36 +2042,52 @@
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Owner Cloudflare action — app project reconnected; crewlogic-marketing still needs Git reconnect.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n">
+      <c r="A44" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Infra / Deploy</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>Retire the last n8n dependency</t>
         </is>
       </c>
-      <c r="D44" s="7" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>Only the route-optimization engine still runs in n8n.</t>
         </is>
       </c>
-      <c r="E44" s="7" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>Retiring it is tied to the Route Optimizer re-architecture.</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr"/>
-      <c r="G44" s="7" t="inlineStr"/>
-      <c r="H44" s="7" t="inlineStr"/>
+      <c r="F44" s="8" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>N8N_BASE + apiFetch('/crewlogic-route') still live (index.html:3962,11598); route engine unchanged on n8n.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -1743,36 +2114,52 @@
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Dual-WRITE shipped (crewlogic-estimate mirrors into estimate_charges); ZERO reads yet + prod-apply 0012/0013 + retire blob remain.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>Infra / Deploy</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>Storage headroom / STORAGE_INCLUDED_GB</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
         <is>
           <t>Prod is on Supabase free tier and the secret isn't set, so the usage dashboard defaults to 1 GB.</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>Set the prod secret to 100 when moving to Supabase Pro; watch estimate-photo storage as testers onboard.</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr"/>
-      <c r="G46" s="7" t="inlineStr"/>
-      <c r="H46" s="7" t="inlineStr"/>
+      <c r="F46" s="8" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Owner action — prod STORAGE_INCLUDED_GB unset (dashboard defaults 1GB); set to 100 on Supabase Pro.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -1799,36 +2186,52 @@
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
-      <c r="H47" s="4" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Upload path already per-franchise; RLS bucket-scoped only (0011) — path-level scoping deferred.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>Rotate + strip committed API keys</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>docs/Route Optimization.json embeds live Google Maps, Anthropic (x2), and Motive keys.</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>Rotate the exposed keys and strip the file (HEAD removal is the ceiling on this private repo).</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr"/>
-      <c r="G48" s="7" t="inlineStr"/>
-      <c r="H48" s="7" t="inlineStr"/>
+      <c r="F48" s="8" t="inlineStr"/>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>File is gitignored + never committed (strip effectively covered); keys NOT rotated — rotation remains.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -1855,36 +2258,52 @@
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Street View still client-side hardcoded STREET_VIEW_KEY (no edge-fn proxy); keys split across projects, no consolidation.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n">
+      <c r="A50" s="7" t="n">
         <v>48</v>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>Track Photo-Analyzer volume-tier adjustments</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>Record when a user bumps an estimate up/down a tier after the AI Photo Analyzer, to measure and correct its bias.</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
         <is>
           <t>Not started; plan first (usage_events vs dedicated table, AI-only scope, store raw suggested CY?).</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr"/>
-      <c r="G50" s="7" t="inlineStr"/>
-      <c r="H50" s="7" t="inlineStr"/>
+      <c r="F50" s="8" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Tier overrides stored client-side only; no analytics event on post-analyzer tier bump.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -1911,36 +2330,52 @@
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>usage.ts emits ai.*/maps.* only; no price.lookup/estimate.created/Street-View metering.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n">
+      <c r="A52" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>Provisioning validation (QA)</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>Live Vonigo-connect prod validation</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>The two @junkluggers.com provisioning cells (invite + marketing) were never run end-to-end in prod.</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
         <is>
           <t>Validate on a real onboarding: user -&gt; Vonigo-pending profile -&gt; enter creds -&gt; franchise attaches under the JL tenant with no paywall (marketing cell carries the 14-day clock).</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr"/>
-      <c r="G52" s="7" t="inlineStr"/>
-      <c r="H52" s="7" t="inlineStr"/>
+      <c r="F52" s="8" t="inlineStr"/>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>Runtime — provisioning cells exist in code; no evidence the 2 @junkluggers.com cells were run end-to-end in prod.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -1967,8 +2402,16 @@
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="4" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>DMARC/SPF/DKIM done; real-signup inbox re-test remains (runtime).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:H53"/>
@@ -1980,7 +2423,7 @@
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not started,In progress,Blocked,Done,Dropped"</formula1>
+      <formula1>"Not started,In progress,Partial,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>